<commit_message>
fixed mutiline chart and added extra data to GOS_SAL_PGR
</commit_message>
<xml_diff>
--- a/Data/GOS_SAL_PGR_ALL_AREA.xlsx
+++ b/Data/GOS_SAL_PGR_ALL_AREA.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\10305\Downloads\Github\FIT3179DV2\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\10305\Downloads\Github\FIT3179DataVisualization2\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C83D2C4F-C858-41BC-8CE4-314351B6921E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D837D7F6-2992-4B87-A93B-1D5570FEB2A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="162">
   <si>
     <t>Postgraduate research median full-time salaries by study area and gender, 2022 and 2023 ($)</t>
   </si>
@@ -319,13 +319,205 @@
   </si>
   <si>
     <t>Total 2021</t>
+  </si>
+  <si>
+    <t>Male 2024</t>
+  </si>
+  <si>
+    <t>126,500</t>
+  </si>
+  <si>
+    <t>115,000</t>
+  </si>
+  <si>
+    <t>106,300</t>
+  </si>
+  <si>
+    <t>114,800</t>
+  </si>
+  <si>
+    <t>90,800</t>
+  </si>
+  <si>
+    <t>143,500</t>
+  </si>
+  <si>
+    <t>110,000</t>
+  </si>
+  <si>
+    <t>97,400</t>
+  </si>
+  <si>
+    <t>122,500</t>
+  </si>
+  <si>
+    <t>106,200</t>
+  </si>
+  <si>
+    <t>23,200</t>
+  </si>
+  <si>
+    <t>Male 2025</t>
+  </si>
+  <si>
+    <t>100,000</t>
+  </si>
+  <si>
+    <t>115,500</t>
+  </si>
+  <si>
+    <t>117,200</t>
+  </si>
+  <si>
+    <t>99,000</t>
+  </si>
+  <si>
+    <t>112,000</t>
+  </si>
+  <si>
+    <t>120,000</t>
+  </si>
+  <si>
+    <t>146,000</t>
+  </si>
+  <si>
+    <t>104,600</t>
+  </si>
+  <si>
+    <t>126,600</t>
+  </si>
+  <si>
+    <t>23,600</t>
+  </si>
+  <si>
+    <t>Female 2024</t>
+  </si>
+  <si>
+    <t>94,400</t>
+  </si>
+  <si>
+    <t>108,500</t>
+  </si>
+  <si>
+    <t>75,000</t>
+  </si>
+  <si>
+    <t>97,000</t>
+  </si>
+  <si>
+    <t>114,300</t>
+  </si>
+  <si>
+    <t>96,600</t>
+  </si>
+  <si>
+    <t>120,900</t>
+  </si>
+  <si>
+    <t>108,000</t>
+  </si>
+  <si>
+    <t>97,500</t>
+  </si>
+  <si>
+    <t>102,000</t>
+  </si>
+  <si>
+    <t>Female 2025</t>
+  </si>
+  <si>
+    <t>104,400</t>
+  </si>
+  <si>
+    <t>104,500</t>
+  </si>
+  <si>
+    <t>112,900</t>
+  </si>
+  <si>
+    <t>130,600</t>
+  </si>
+  <si>
+    <t>106,000</t>
+  </si>
+  <si>
+    <t>123,000</t>
+  </si>
+  <si>
+    <t>107,100</t>
+  </si>
+  <si>
+    <t>14,500</t>
+  </si>
+  <si>
+    <t>Total 2024</t>
+  </si>
+  <si>
+    <t>95,800</t>
+  </si>
+  <si>
+    <t>123,500</t>
+  </si>
+  <si>
+    <t>89,500</t>
+  </si>
+  <si>
+    <t>105,300</t>
+  </si>
+  <si>
+    <t>114,700</t>
+  </si>
+  <si>
+    <t>93,600</t>
+  </si>
+  <si>
+    <t>93,000</t>
+  </si>
+  <si>
+    <t>13,800</t>
+  </si>
+  <si>
+    <t>Total 2025</t>
+  </si>
+  <si>
+    <t>98,700</t>
+  </si>
+  <si>
+    <t>110,100</t>
+  </si>
+  <si>
+    <t>109,000</t>
+  </si>
+  <si>
+    <t>103,000</t>
+  </si>
+  <si>
+    <t>125,500</t>
+  </si>
+  <si>
+    <t>116,000</t>
+  </si>
+  <si>
+    <t>132,000</t>
+  </si>
+  <si>
+    <t>107,500</t>
+  </si>
+  <si>
+    <t>124,500</t>
+  </si>
+  <si>
+    <t>109,100</t>
+  </si>
+  <si>
+    <t>21,400</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -350,6 +542,12 @@
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -364,7 +562,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -396,11 +594,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="thick">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -410,8 +619,11 @@
     <xf numFmtId="3" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -720,11 +932,16 @@
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
     </row>
-    <row r="2" spans="1:20" ht="25.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:20" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="B2" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>98</v>
+      </c>
       <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
@@ -737,8 +954,12 @@
       <c r="G2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
+      <c r="H2" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>121</v>
+      </c>
       <c r="J2" s="4" t="s">
         <v>5</v>
       </c>
@@ -751,8 +972,12 @@
       <c r="M2" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
+      <c r="N2" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="O2" s="7" t="s">
+        <v>141</v>
+      </c>
       <c r="P2" s="4" t="s">
         <v>7</v>
       </c>
@@ -771,7 +996,12 @@
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2"/>
+      <c r="B3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
       <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
@@ -784,8 +1014,12 @@
       <c r="G3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="H3" t="s">
+        <v>125</v>
+      </c>
+      <c r="I3" t="s">
+        <v>122</v>
+      </c>
       <c r="J3" s="2" t="s">
         <v>12</v>
       </c>
@@ -798,8 +1032,12 @@
       <c r="M3" s="2">
         <v>84900</v>
       </c>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
+      <c r="N3" t="s">
+        <v>151</v>
+      </c>
+      <c r="O3" t="s">
+        <v>142</v>
+      </c>
       <c r="P3" s="2" t="s">
         <v>14</v>
       </c>
@@ -818,7 +1056,12 @@
       <c r="A4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="2"/>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
       <c r="D4" s="2" t="s">
         <v>9</v>
       </c>
@@ -831,8 +1074,12 @@
       <c r="G4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+      <c r="H4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" t="s">
+        <v>9</v>
+      </c>
       <c r="J4" s="2" t="s">
         <v>9</v>
       </c>
@@ -845,8 +1092,12 @@
       <c r="M4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
+      <c r="N4" t="s">
+        <v>9</v>
+      </c>
+      <c r="O4" t="s">
+        <v>9</v>
+      </c>
       <c r="P4" s="2" t="s">
         <v>9</v>
       </c>
@@ -865,7 +1116,12 @@
       <c r="A5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="2"/>
+      <c r="B5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C5" t="s">
+        <v>99</v>
+      </c>
       <c r="D5" s="2" t="s">
         <v>18</v>
       </c>
@@ -878,8 +1134,12 @@
       <c r="G5" s="2">
         <v>105000</v>
       </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
+      <c r="H5" t="s">
+        <v>123</v>
+      </c>
+      <c r="I5" t="s">
+        <v>123</v>
+      </c>
       <c r="J5" s="2" t="s">
         <v>20</v>
       </c>
@@ -892,8 +1152,12 @@
       <c r="M5" s="2">
         <v>97600</v>
       </c>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
+      <c r="N5" t="s">
+        <v>152</v>
+      </c>
+      <c r="O5" t="s">
+        <v>143</v>
+      </c>
       <c r="P5" s="2" t="s">
         <v>22</v>
       </c>
@@ -912,7 +1176,12 @@
       <c r="A6" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="2"/>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
       <c r="D6" s="2" t="s">
         <v>9</v>
       </c>
@@ -925,8 +1194,12 @@
       <c r="G6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
+      <c r="H6" t="s">
+        <v>9</v>
+      </c>
+      <c r="I6" t="s">
+        <v>9</v>
+      </c>
       <c r="J6" s="2" t="s">
         <v>9</v>
       </c>
@@ -939,8 +1212,12 @@
       <c r="M6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
+      <c r="N6" t="s">
+        <v>9</v>
+      </c>
+      <c r="O6" t="s">
+        <v>9</v>
+      </c>
       <c r="P6" s="2" t="s">
         <v>9</v>
       </c>
@@ -959,7 +1236,12 @@
       <c r="A7" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="B7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C7" t="s">
+        <v>100</v>
+      </c>
       <c r="D7" s="2" t="s">
         <v>26</v>
       </c>
@@ -972,8 +1254,12 @@
       <c r="G7" s="2">
         <v>92000</v>
       </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="H7" t="s">
+        <v>9</v>
+      </c>
+      <c r="I7" t="s">
+        <v>9</v>
+      </c>
       <c r="J7" s="2" t="s">
         <v>9</v>
       </c>
@@ -986,8 +1272,12 @@
       <c r="M7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
+      <c r="N7" t="s">
+        <v>153</v>
+      </c>
+      <c r="O7" t="s">
+        <v>123</v>
+      </c>
       <c r="P7" s="2" t="s">
         <v>26</v>
       </c>
@@ -1006,7 +1296,12 @@
       <c r="A8" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="B8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
       <c r="D8" s="2" t="s">
         <v>30</v>
       </c>
@@ -1019,8 +1314,12 @@
       <c r="G8" s="2">
         <v>93000</v>
       </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="H8" t="s">
+        <v>133</v>
+      </c>
+      <c r="I8" t="s">
+        <v>124</v>
+      </c>
       <c r="J8" s="2" t="s">
         <v>32</v>
       </c>
@@ -1033,8 +1332,12 @@
       <c r="M8" s="2">
         <v>70000</v>
       </c>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
+      <c r="N8" t="s">
+        <v>154</v>
+      </c>
+      <c r="O8" t="s">
+        <v>144</v>
+      </c>
       <c r="P8" s="2" t="s">
         <v>34</v>
       </c>
@@ -1053,7 +1356,12 @@
       <c r="A9" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="2"/>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
       <c r="D9" s="2" t="s">
         <v>9</v>
       </c>
@@ -1066,8 +1374,12 @@
       <c r="G9" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="H9" t="s">
+        <v>9</v>
+      </c>
+      <c r="I9" t="s">
+        <v>9</v>
+      </c>
       <c r="J9" s="2" t="s">
         <v>1</v>
       </c>
@@ -1080,8 +1392,12 @@
       <c r="M9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
+      <c r="N9" t="s">
+        <v>9</v>
+      </c>
+      <c r="O9" t="s">
+        <v>9</v>
+      </c>
       <c r="P9" s="2" t="s">
         <v>1</v>
       </c>
@@ -1100,7 +1416,12 @@
       <c r="A10" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="2"/>
+      <c r="B10" t="s">
+        <v>115</v>
+      </c>
+      <c r="C10" t="s">
+        <v>101</v>
+      </c>
       <c r="D10" s="2" t="s">
         <v>38</v>
       </c>
@@ -1113,8 +1434,12 @@
       <c r="G10" s="2">
         <v>93900</v>
       </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
+      <c r="H10" t="s">
+        <v>134</v>
+      </c>
+      <c r="I10" t="s">
+        <v>125</v>
+      </c>
       <c r="J10" s="2" t="s">
         <v>40</v>
       </c>
@@ -1127,8 +1452,12 @@
       <c r="M10" s="2">
         <v>90800</v>
       </c>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
+      <c r="N10" t="s">
+        <v>105</v>
+      </c>
+      <c r="O10" t="s">
+        <v>145</v>
+      </c>
       <c r="P10" s="2" t="s">
         <v>41</v>
       </c>
@@ -1147,7 +1476,12 @@
       <c r="A11" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="2"/>
+      <c r="B11" t="s">
+        <v>116</v>
+      </c>
+      <c r="C11" t="s">
+        <v>102</v>
+      </c>
       <c r="D11" s="2" t="s">
         <v>44</v>
       </c>
@@ -1160,8 +1494,12 @@
       <c r="G11" s="2">
         <v>98600</v>
       </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
+      <c r="H11" t="s">
+        <v>135</v>
+      </c>
+      <c r="I11" t="s">
+        <v>126</v>
+      </c>
       <c r="J11" s="2" t="s">
         <v>46</v>
       </c>
@@ -1174,8 +1512,12 @@
       <c r="M11" s="2">
         <v>93500</v>
       </c>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
+      <c r="N11" t="s">
+        <v>112</v>
+      </c>
+      <c r="O11" t="s">
+        <v>146</v>
+      </c>
       <c r="P11" s="2" t="s">
         <v>21</v>
       </c>
@@ -1194,7 +1536,12 @@
       <c r="A12" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" t="s">
+        <v>103</v>
+      </c>
       <c r="D12" s="2" t="s">
         <v>48</v>
       </c>
@@ -1207,8 +1554,12 @@
       <c r="G12" s="2">
         <v>90000</v>
       </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="H12" t="s">
+        <v>111</v>
+      </c>
+      <c r="I12" t="s">
+        <v>127</v>
+      </c>
       <c r="J12" s="2" t="s">
         <v>50</v>
       </c>
@@ -1221,8 +1572,12 @@
       <c r="M12" s="2">
         <v>90000</v>
       </c>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
+      <c r="N12" t="s">
+        <v>129</v>
+      </c>
+      <c r="O12" t="s">
+        <v>147</v>
+      </c>
       <c r="P12" s="2" t="s">
         <v>51</v>
       </c>
@@ -1241,7 +1596,12 @@
       <c r="A13" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="2"/>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
       <c r="D13" s="2" t="s">
         <v>9</v>
       </c>
@@ -1254,8 +1614,12 @@
       <c r="G13" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
+      <c r="H13" t="s">
+        <v>9</v>
+      </c>
+      <c r="I13" t="s">
+        <v>9</v>
+      </c>
       <c r="J13" s="2" t="s">
         <v>9</v>
       </c>
@@ -1268,8 +1632,12 @@
       <c r="M13" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
+      <c r="N13" t="s">
+        <v>155</v>
+      </c>
+      <c r="O13" t="s">
+        <v>100</v>
+      </c>
       <c r="P13" s="2" t="s">
         <v>54</v>
       </c>
@@ -1288,7 +1656,12 @@
       <c r="A14" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="2"/>
+      <c r="B14" t="s">
+        <v>117</v>
+      </c>
+      <c r="C14" t="s">
+        <v>104</v>
+      </c>
       <c r="D14" s="2" t="s">
         <v>57</v>
       </c>
@@ -1301,8 +1674,12 @@
       <c r="G14" s="2">
         <v>122500</v>
       </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
+      <c r="H14" t="s">
+        <v>105</v>
+      </c>
+      <c r="I14" t="s">
+        <v>105</v>
+      </c>
       <c r="J14" s="2" t="s">
         <v>58</v>
       </c>
@@ -1315,8 +1692,12 @@
       <c r="M14" s="2">
         <v>96300</v>
       </c>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
+      <c r="N14" t="s">
+        <v>156</v>
+      </c>
+      <c r="O14" t="s">
+        <v>100</v>
+      </c>
       <c r="P14" s="2" t="s">
         <v>60</v>
       </c>
@@ -1335,7 +1716,12 @@
       <c r="A15" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="2"/>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
       <c r="D15" s="2" t="s">
         <v>9</v>
       </c>
@@ -1348,8 +1734,12 @@
       <c r="G15" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
+      <c r="H15" t="s">
+        <v>136</v>
+      </c>
+      <c r="I15" t="s">
+        <v>128</v>
+      </c>
       <c r="J15" s="2" t="s">
         <v>63</v>
       </c>
@@ -1362,8 +1752,12 @@
       <c r="M15" s="2">
         <v>109000</v>
       </c>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
+      <c r="N15" t="s">
+        <v>157</v>
+      </c>
+      <c r="O15" t="s">
+        <v>138</v>
+      </c>
       <c r="P15" s="2" t="s">
         <v>64</v>
       </c>
@@ -1382,7 +1776,12 @@
       <c r="A16" t="s">
         <v>65</v>
       </c>
-      <c r="C16" s="2"/>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
+        <v>9</v>
+      </c>
       <c r="D16" s="2" t="s">
         <v>9</v>
       </c>
@@ -1395,8 +1794,12 @@
       <c r="G16" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
+      <c r="H16" t="s">
+        <v>9</v>
+      </c>
+      <c r="I16" t="s">
+        <v>9</v>
+      </c>
       <c r="J16" s="2" t="s">
         <v>9</v>
       </c>
@@ -1409,8 +1812,12 @@
       <c r="M16" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
+      <c r="N16" t="s">
+        <v>9</v>
+      </c>
+      <c r="O16" t="s">
+        <v>148</v>
+      </c>
       <c r="P16" s="2" t="s">
         <v>9</v>
       </c>
@@ -1429,7 +1836,12 @@
       <c r="A17" t="s">
         <v>66</v>
       </c>
-      <c r="C17" s="2"/>
+      <c r="B17" t="s">
+        <v>105</v>
+      </c>
+      <c r="C17" t="s">
+        <v>105</v>
+      </c>
       <c r="D17" s="2" t="s">
         <v>67</v>
       </c>
@@ -1442,8 +1854,12 @@
       <c r="G17" s="2">
         <v>99300</v>
       </c>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
+      <c r="H17" t="s">
+        <v>137</v>
+      </c>
+      <c r="I17" t="s">
+        <v>129</v>
+      </c>
       <c r="J17" s="2" t="s">
         <v>27</v>
       </c>
@@ -1456,8 +1872,12 @@
       <c r="M17" s="2">
         <v>94000</v>
       </c>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
+      <c r="N17" t="s">
+        <v>158</v>
+      </c>
+      <c r="O17" t="s">
+        <v>129</v>
+      </c>
       <c r="P17" s="2" t="s">
         <v>39</v>
       </c>
@@ -1476,7 +1896,12 @@
       <c r="A18" t="s">
         <v>70</v>
       </c>
-      <c r="C18" s="2"/>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
       <c r="D18" s="2" t="s">
         <v>9</v>
       </c>
@@ -1489,8 +1914,12 @@
       <c r="G18" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
+      <c r="H18" t="s">
+        <v>9</v>
+      </c>
+      <c r="I18" t="s">
+        <v>9</v>
+      </c>
       <c r="J18" s="2" t="s">
         <v>9</v>
       </c>
@@ -1503,8 +1932,12 @@
       <c r="M18" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
+      <c r="N18" t="s">
+        <v>9</v>
+      </c>
+      <c r="O18" t="s">
+        <v>9</v>
+      </c>
       <c r="P18" s="2" t="s">
         <v>9</v>
       </c>
@@ -1523,7 +1956,12 @@
       <c r="A19" t="s">
         <v>71</v>
       </c>
-      <c r="C19" s="2"/>
+      <c r="B19" t="s">
+        <v>118</v>
+      </c>
+      <c r="C19" t="s">
+        <v>106</v>
+      </c>
       <c r="D19" s="2" t="s">
         <v>39</v>
       </c>
@@ -1536,8 +1974,12 @@
       <c r="G19" s="2">
         <v>87700</v>
       </c>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
+      <c r="H19" t="s">
+        <v>111</v>
+      </c>
+      <c r="I19" t="s">
+        <v>130</v>
+      </c>
       <c r="J19" s="2" t="s">
         <v>30</v>
       </c>
@@ -1550,8 +1992,12 @@
       <c r="M19" s="2">
         <v>85200</v>
       </c>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2"/>
+      <c r="N19" t="s">
+        <v>131</v>
+      </c>
+      <c r="O19" t="s">
+        <v>130</v>
+      </c>
       <c r="P19" s="2" t="s">
         <v>74</v>
       </c>
@@ -1570,7 +2016,12 @@
       <c r="A20" t="s">
         <v>75</v>
       </c>
-      <c r="C20" s="2"/>
+      <c r="B20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
+        <v>1</v>
+      </c>
       <c r="D20" s="2" t="s">
         <v>9</v>
       </c>
@@ -1583,8 +2034,12 @@
       <c r="G20" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
+      <c r="H20" t="s">
+        <v>9</v>
+      </c>
+      <c r="I20" t="s">
+        <v>9</v>
+      </c>
       <c r="J20" s="2" t="s">
         <v>9</v>
       </c>
@@ -1597,8 +2052,12 @@
       <c r="M20" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
+      <c r="N20" t="s">
+        <v>9</v>
+      </c>
+      <c r="O20" t="s">
+        <v>9</v>
+      </c>
       <c r="P20" s="2" t="s">
         <v>9</v>
       </c>
@@ -1617,7 +2076,12 @@
       <c r="A21" t="s">
         <v>76</v>
       </c>
-      <c r="C21" s="2"/>
+      <c r="B21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21" t="s">
+        <v>107</v>
+      </c>
       <c r="D21" s="2" t="s">
         <v>78</v>
       </c>
@@ -1630,8 +2094,12 @@
       <c r="G21" s="2">
         <v>120000</v>
       </c>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
+      <c r="H21" t="s">
+        <v>138</v>
+      </c>
+      <c r="I21" t="s">
+        <v>116</v>
+      </c>
       <c r="J21" s="2" t="s">
         <v>80</v>
       </c>
@@ -1644,8 +2112,12 @@
       <c r="M21" s="2">
         <v>110000</v>
       </c>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
+      <c r="N21" t="s">
+        <v>159</v>
+      </c>
+      <c r="O21" t="s">
+        <v>116</v>
+      </c>
       <c r="P21" s="2" t="s">
         <v>80</v>
       </c>
@@ -1664,7 +2136,12 @@
       <c r="A22" t="s">
         <v>81</v>
       </c>
-      <c r="C22" s="2"/>
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" t="s">
+        <v>1</v>
+      </c>
       <c r="D22" s="2" t="s">
         <v>9</v>
       </c>
@@ -1677,8 +2154,12 @@
       <c r="G22" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
+      <c r="H22" t="s">
+        <v>1</v>
+      </c>
+      <c r="I22" t="s">
+        <v>1</v>
+      </c>
       <c r="J22" s="2" t="s">
         <v>1</v>
       </c>
@@ -1691,8 +2172,12 @@
       <c r="M22" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
+      <c r="N22" t="s">
+        <v>9</v>
+      </c>
+      <c r="O22" t="s">
+        <v>1</v>
+      </c>
       <c r="P22" s="2" t="s">
         <v>9</v>
       </c>
@@ -1711,7 +2196,12 @@
       <c r="A23" t="s">
         <v>82</v>
       </c>
-      <c r="C23" s="2"/>
+      <c r="B23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" t="s">
+        <v>9</v>
+      </c>
       <c r="D23" s="2" t="s">
         <v>9</v>
       </c>
@@ -1724,8 +2214,12 @@
       <c r="G23" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
+      <c r="H23" t="s">
+        <v>9</v>
+      </c>
+      <c r="I23" t="s">
+        <v>9</v>
+      </c>
       <c r="J23" s="2" t="s">
         <v>9</v>
       </c>
@@ -1738,8 +2232,12 @@
       <c r="M23" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2"/>
+      <c r="N23" t="s">
+        <v>9</v>
+      </c>
+      <c r="O23" t="s">
+        <v>9</v>
+      </c>
       <c r="P23" s="2" t="s">
         <v>9</v>
       </c>
@@ -1758,7 +2256,12 @@
       <c r="A24" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C24" s="1"/>
+      <c r="B24" t="s">
+        <v>115</v>
+      </c>
+      <c r="C24" t="s">
+        <v>108</v>
+      </c>
       <c r="D24" s="1" t="s">
         <v>38</v>
       </c>
@@ -1771,8 +2274,12 @@
       <c r="G24" s="1">
         <v>95000</v>
       </c>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
+      <c r="H24" t="s">
+        <v>139</v>
+      </c>
+      <c r="I24" t="s">
+        <v>131</v>
+      </c>
       <c r="J24" s="1" t="s">
         <v>50</v>
       </c>
@@ -1785,8 +2292,12 @@
       <c r="M24" s="1">
         <v>91900</v>
       </c>
-      <c r="N24" s="1"/>
-      <c r="O24" s="1"/>
+      <c r="N24" t="s">
+        <v>160</v>
+      </c>
+      <c r="O24" t="s">
+        <v>133</v>
+      </c>
       <c r="P24" s="1" t="s">
         <v>38</v>
       </c>
@@ -1805,6 +2316,12 @@
       <c r="A25" t="s">
         <v>85</v>
       </c>
+      <c r="B25" t="s">
+        <v>120</v>
+      </c>
+      <c r="C25" t="s">
+        <v>109</v>
+      </c>
       <c r="D25" t="s">
         <v>87</v>
       </c>
@@ -1817,6 +2334,12 @@
       <c r="G25">
         <v>13900</v>
       </c>
+      <c r="H25" t="s">
+        <v>140</v>
+      </c>
+      <c r="I25" t="s">
+        <v>90</v>
+      </c>
       <c r="J25" t="s">
         <v>89</v>
       </c>
@@ -1828,6 +2351,12 @@
       </c>
       <c r="M25">
         <v>10800</v>
+      </c>
+      <c r="N25" t="s">
+        <v>161</v>
+      </c>
+      <c r="O25" t="s">
+        <v>149</v>
       </c>
       <c r="P25" t="s">
         <v>91</v>

</xml_diff>